<commit_message>
feat: expand cultivation and item progression
</commit_message>
<xml_diff>
--- a/config/xlsx/game_config.xlsx
+++ b/config/xlsx/game_config.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -498,30 +498,50 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>reset_hour</t>
+          <t>stamina.multiplier_threshold_base</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>craft_speedup_stone_cost_per_minute</t>
+          <t>stamina.multiplier_duration</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>1</v>
+        <v>3600</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>reset_hour</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>craft_speedup_stone_cost_per_minute</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>launcher_speedup_stone_cost_per_minute</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B10" s="2" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>